<commit_message>
feat(procurement): enhance MTS and PO tracking with complete lifecycle timeline and KPIs
</commit_message>
<xml_diff>
--- a/sample_output/Horizon_Smart_Tower_Daily_Schedule.xlsx
+++ b/sample_output/Horizon_Smart_Tower_Daily_Schedule.xlsx
@@ -516,7 +516,7 @@
         <v>إجمالي المهام المجدولة:</v>
       </c>
       <c r="B14">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15">
@@ -524,7 +524,7 @@
         <v>المهام المكتملة:</v>
       </c>
       <c r="B15">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -532,7 +532,7 @@
         <v>المهام الجاري تنفيذها:</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -540,7 +540,7 @@
         <v>المهام المعلقة / المخططة:</v>
       </c>
       <c r="B17">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -548,7 +548,7 @@
         <v>المهام ذات الأولوية الحرجة (Critical):</v>
       </c>
       <c r="B18">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19">
@@ -556,7 +556,7 @@
         <v>نسبة الإنجاز العامة المخططة:</v>
       </c>
       <c r="B19" t="str">
-        <v>35%</v>
+        <v>38%</v>
       </c>
     </row>
     <row r="20">
@@ -648,7 +648,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L61"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -707,7 +707,7 @@
         <v>TSK-0001</v>
       </c>
       <c r="B2" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-01</v>
       </c>
       <c r="C2" t="str">
         <v>Mobilization &amp; Kick-off</v>
@@ -716,16 +716,16 @@
         <v>Management</v>
       </c>
       <c r="E2" t="str">
-        <v>عقد اجتماع انطلاق المشروع (Kick-off Meeting) وتوزيع مصفوفة الصلاحيات (RACI)</v>
+        <v>عقد الاجتماع التنسيقي لانطلاق مشروع: مشروع برج الأفق الذكي للأعمال والفندقة واعتماد خطة العمل</v>
       </c>
       <c r="F2" t="str">
-        <v>Conduct Project Kick-off Meeting &amp; Establish RACI Matrix</v>
+        <v>Conduct Project Kick-off Meeting for: Horizon Smart Business Tower &amp; Luxury Suites &amp; Finalize Project Management Plan</v>
       </c>
       <c r="G2" t="str">
         <v>Project Manager</v>
       </c>
       <c r="H2" t="str">
-        <v>General</v>
+        <v>General / عام</v>
       </c>
       <c r="I2" t="str">
         <v>Critical</v>
@@ -737,7 +737,7 @@
         <v>100%</v>
       </c>
       <c r="L2" t="str">
-        <v>Kick-off Presentation &amp; Signed Minutes of Meeting</v>
+        <v>Signed Kick-off Minutes &amp; Project Charter</v>
       </c>
     </row>
     <row r="3">
@@ -745,25 +745,25 @@
         <v>TSK-0002</v>
       </c>
       <c r="B3" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-01</v>
       </c>
       <c r="C3" t="str">
-        <v>Mobilization &amp; Kick-off</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D3" t="str">
-        <v>Engineering</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E3" t="str">
-        <v>استلام ومراجعة مستندات ومخططات الـ IFC الأولية لنظام شبكات الـ ICT و التيار الخفيف</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: انطلاق المشروع والتهيئة الميدانية (Project Mobilization)</v>
       </c>
       <c r="F3" t="str">
-        <v>Review initial IFC drawings for ICT and ELV systems</v>
+        <v>Commence activities for milestone: انطلاق المشروع والتهيئة الميدانية (Project Mobilization)</v>
       </c>
       <c r="G3" t="str">
-        <v>Technical Manager</v>
+        <v>Project Manager</v>
       </c>
       <c r="H3" t="str">
-        <v>General</v>
+        <v>Project Site</v>
       </c>
       <c r="I3" t="str">
         <v>High</v>
@@ -775,7 +775,7 @@
         <v>100%</v>
       </c>
       <c r="L3" t="str">
-        <v>IFC Review Log &amp; Design Queries</v>
+        <v>Milestone Commencement Transmittal (5%)</v>
       </c>
     </row>
     <row r="4">
@@ -783,37 +783,37 @@
         <v>TSK-0003</v>
       </c>
       <c r="B4" t="str">
-        <v>2025-09-25</v>
+        <v>2025-11-15</v>
       </c>
       <c r="C4" t="str">
-        <v>Mobilization &amp; Kick-off</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D4" t="str">
-        <v>Procurement</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E4" t="str">
-        <v>حصر الموردين المعتمدين (Vendor List) وتجهيز طلبات التأهيل المسبق (Prequalifications)</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: المخططات الهندسية واعتمادات المواد (MTS Approvals)</v>
       </c>
       <c r="F4" t="str">
-        <v>Prepare Approved Vendor List and vendor prequalification packages</v>
+        <v>Commence activities for milestone: المخططات الهندسية واعتمادات المواد (MTS Approvals)</v>
       </c>
       <c r="G4" t="str">
-        <v>Procurement Manager</v>
+        <v>Technical Manager</v>
       </c>
       <c r="H4" t="str">
-        <v>General</v>
+        <v>Project Site</v>
       </c>
       <c r="I4" t="str">
         <v>High</v>
       </c>
       <c r="J4" t="str">
-        <v>Completed</v>
+        <v>In Progress</v>
       </c>
       <c r="K4" t="str">
-        <v>100%</v>
+        <v>50%</v>
       </c>
       <c r="L4" t="str">
-        <v>Vendor List &amp; Pre-qual Submissions</v>
+        <v>Milestone Commencement Transmittal (20%)</v>
       </c>
     </row>
     <row r="5">
@@ -821,37 +821,37 @@
         <v>TSK-0004</v>
       </c>
       <c r="B5" t="str">
-        <v>2025-10-05</v>
+        <v>2025-12-01</v>
       </c>
       <c r="C5" t="str">
-        <v>Mobilization &amp; Kick-off</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D5" t="str">
-        <v>Planning</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E5" t="str">
-        <v>إعداد خطة إدارة المشروع (PMP) والجدول الزمني التمهيدي على Primavera</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: نمذجة معلومات البناء وتنسيق BIM (BIM Coordination)</v>
       </c>
       <c r="F5" t="str">
-        <v>Develop Project Management Plan (PMP) &amp; Primavera Baseline Schedule</v>
+        <v>Commence activities for milestone: نمذجة معلومات البناء وتنسيق BIM (BIM Coordination)</v>
       </c>
       <c r="G5" t="str">
-        <v>Planning Manager</v>
+        <v>BIM Lead</v>
       </c>
       <c r="H5" t="str">
-        <v>General</v>
+        <v>Project Site</v>
       </c>
       <c r="I5" t="str">
-        <v>Critical</v>
+        <v>High</v>
       </c>
       <c r="J5" t="str">
-        <v>Completed</v>
+        <v>In Progress</v>
       </c>
       <c r="K5" t="str">
-        <v>100%</v>
+        <v>50%</v>
       </c>
       <c r="L5" t="str">
-        <v>Approved Baseline Schedule Rev00</v>
+        <v>Milestone Commencement Transmittal (10%)</v>
       </c>
     </row>
     <row r="6">
@@ -859,28 +859,28 @@
         <v>TSK-0005</v>
       </c>
       <c r="B6" t="str">
-        <v>2025-10-15</v>
+        <v>2025-12-20</v>
       </c>
       <c r="C6" t="str">
-        <v>Mobilization &amp; Kick-off</v>
+        <v>Milestone Completion</v>
       </c>
       <c r="D6" t="str">
-        <v>HSE &amp; QA/QC</v>
+        <v>QA/QC &amp; Delivery</v>
       </c>
       <c r="E6" t="str">
-        <v>تقديم خطة السلامة والصحة المهنية (HSE Plan) وخطة ضبط الجودة (QA/QC Plan)</v>
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: انطلاق المشروع والتهيئة الميدانية (Project Mobilization)</v>
       </c>
       <c r="F6" t="str">
-        <v>Submit Site HSE Plan and QA/QC Project Quality Plan (PQP)</v>
+        <v>Finalize and deliver outputs for milestone: انطلاق المشروع والتهيئة الميدانية (Project Mobilization)</v>
       </c>
       <c r="G6" t="str">
-        <v>HSE Manager</v>
+        <v>Project Manager</v>
       </c>
       <c r="H6" t="str">
-        <v>General</v>
+        <v>Project Site</v>
       </c>
       <c r="I6" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J6" t="str">
         <v>Completed</v>
@@ -889,7 +889,7 @@
         <v>100%</v>
       </c>
       <c r="L6" t="str">
-        <v>Approved HSE &amp; QA/QC Plans</v>
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
       </c>
     </row>
     <row r="7">
@@ -900,22 +900,22 @@
         <v>2026-01-05</v>
       </c>
       <c r="C7" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D7" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E7" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
       </c>
       <c r="F7" t="str">
-        <v>Submit Material Submittal (MTS) for: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
+        <v>Submit Material Submittal &amp; Compliance for: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
       </c>
       <c r="G7" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H7" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I7" t="str">
         <v>High</v>
@@ -927,7 +927,7 @@
         <v>100%</v>
       </c>
       <c r="L7" t="str">
-        <v>MTS Document Package (Status: A - Approved)</v>
+        <v>MTS Package (Status Code: A)</v>
       </c>
     </row>
     <row r="8">
@@ -938,22 +938,22 @@
         <v>2026-01-15</v>
       </c>
       <c r="C8" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D8" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E8" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
       </c>
       <c r="F8" t="str">
-        <v>Submit Material Submittal (MTS) for: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
+        <v>Submit Material Submittal &amp; Compliance for: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
       </c>
       <c r="G8" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H8" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I8" t="str">
         <v>Critical</v>
@@ -965,7 +965,7 @@
         <v>100%</v>
       </c>
       <c r="L8" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="9">
@@ -976,22 +976,22 @@
         <v>2026-01-20</v>
       </c>
       <c r="C9" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D9" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E9" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
       </c>
       <c r="F9" t="str">
-        <v>Submit Material Submittal (MTS) for: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
+        <v>Submit Material Submittal &amp; Compliance for: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
       </c>
       <c r="G9" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H9" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I9" t="str">
         <v>Critical</v>
@@ -1003,7 +1003,7 @@
         <v>100%</v>
       </c>
       <c r="L9" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="10">
@@ -1011,28 +1011,28 @@
         <v>TSK-0009</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-02-10</v>
+        <v>2026-02-01</v>
       </c>
       <c r="C10" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D10" t="str">
-        <v>MTS Submittal</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E10" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
       </c>
       <c r="F10" t="str">
-        <v>Submit Material Submittal (MTS) for: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
       </c>
       <c r="G10" t="str">
-        <v>Technical Manager</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H10" t="str">
-        <v>General</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I10" t="str">
-        <v>Critical</v>
+        <v>High</v>
       </c>
       <c r="J10" t="str">
         <v>Completed</v>
@@ -1041,7 +1041,7 @@
         <v>100%</v>
       </c>
       <c r="L10" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="11">
@@ -1049,25 +1049,25 @@
         <v>TSK-0010</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-02-22</v>
+        <v>2026-02-10</v>
       </c>
       <c r="C11" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D11" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E11" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
       </c>
       <c r="F11" t="str">
-        <v>Submit Material Submittal (MTS) for: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
+        <v>Submit Material Submittal &amp; Compliance for: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
       </c>
       <c r="G11" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H11" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I11" t="str">
         <v>Critical</v>
@@ -1079,7 +1079,7 @@
         <v>100%</v>
       </c>
       <c r="L11" t="str">
-        <v>MTS Document Package (Status: C - Revise &amp; Resubmit)</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="12">
@@ -1087,37 +1087,37 @@
         <v>TSK-0011</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-02-28</v>
+        <v>2026-02-22</v>
       </c>
       <c r="C12" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D12" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E12" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
       </c>
       <c r="F12" t="str">
-        <v>Submit Material Submittal (MTS) for: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
+        <v>Submit Material Submittal &amp; Compliance for: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
       </c>
       <c r="G12" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H12" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I12" t="str">
         <v>Critical</v>
       </c>
       <c r="J12" t="str">
-        <v>Completed</v>
+        <v>In Progress</v>
       </c>
       <c r="K12" t="str">
-        <v>100%</v>
+        <v>40%</v>
       </c>
       <c r="L12" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>MTS Package (Status Code: C)</v>
       </c>
     </row>
     <row r="13">
@@ -1125,25 +1125,25 @@
         <v>TSK-0012</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-03-05</v>
+        <v>2026-02-28</v>
       </c>
       <c r="C13" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D13" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E13" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
       </c>
       <c r="F13" t="str">
-        <v>Submit Material Submittal (MTS) for: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
+        <v>Submit Material Submittal &amp; Compliance for: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
       </c>
       <c r="G13" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H13" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I13" t="str">
         <v>Critical</v>
@@ -1155,7 +1155,7 @@
         <v>100%</v>
       </c>
       <c r="L13" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="14">
@@ -1163,37 +1163,37 @@
         <v>TSK-0013</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-03-18</v>
+        <v>2026-03-01</v>
       </c>
       <c r="C14" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D14" t="str">
-        <v>MTS Submittal</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E14" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: إصدار أوامر الشراء للمواد طويلة التوريد (Procurement Long-Lead POs)</v>
       </c>
       <c r="F14" t="str">
-        <v>Submit Material Submittal (MTS) for: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
+        <v>Commence activities for milestone: إصدار أوامر الشراء للمواد طويلة التوريد (Procurement Long-Lead POs)</v>
       </c>
       <c r="G14" t="str">
-        <v>Technical Manager</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H14" t="str">
-        <v>General</v>
+        <v>Project Site</v>
       </c>
       <c r="I14" t="str">
         <v>Critical</v>
       </c>
       <c r="J14" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="K14" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
       <c r="L14" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>Milestone Commencement Transmittal (20%)</v>
       </c>
     </row>
     <row r="15">
@@ -1201,28 +1201,28 @@
         <v>TSK-0014</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-04-10</v>
+        <v>2026-03-05</v>
       </c>
       <c r="C15" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D15" t="str">
-        <v>MTS Submittal</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E15" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
       </c>
       <c r="F15" t="str">
-        <v>Submit Material Submittal (MTS) for: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
       </c>
       <c r="G15" t="str">
-        <v>Technical Manager</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H15" t="str">
-        <v>General</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I15" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J15" t="str">
         <v>Completed</v>
@@ -1231,7 +1231,7 @@
         <v>100%</v>
       </c>
       <c r="L15" t="str">
-        <v>MTS Document Package (Status: C - Revise &amp; Resubmit)</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="16">
@@ -1239,25 +1239,25 @@
         <v>TSK-0015</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-04-15</v>
+        <v>2026-03-05</v>
       </c>
       <c r="C16" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D16" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E16" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
       </c>
       <c r="F16" t="str">
-        <v>Submit Material Submittal (MTS) for: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
+        <v>Submit Material Submittal &amp; Compliance for: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
       </c>
       <c r="G16" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H16" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I16" t="str">
         <v>Critical</v>
@@ -1269,7 +1269,7 @@
         <v>100%</v>
       </c>
       <c r="L16" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="17">
@@ -1277,25 +1277,25 @@
         <v>TSK-0016</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-05-12</v>
+        <v>2026-03-08</v>
       </c>
       <c r="C17" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D17" t="str">
-        <v>MTS Submittal</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E17" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
       </c>
       <c r="F17" t="str">
-        <v>Submit Material Submittal (MTS) for: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
       </c>
       <c r="G17" t="str">
-        <v>Technical Manager</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H17" t="str">
-        <v>General</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I17" t="str">
         <v>Critical</v>
@@ -1307,7 +1307,7 @@
         <v>100%</v>
       </c>
       <c r="L17" t="str">
-        <v>MTS Document Package (Status: B - Approved as Noted)</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="18">
@@ -1315,25 +1315,25 @@
         <v>TSK-0017</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-05-20</v>
+        <v>2026-03-18</v>
       </c>
       <c r="C18" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D18" t="str">
-        <v>MTS Submittal</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E18" t="str">
-        <v>تقديم اعتماد المواد (MTS) لنظام: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
       </c>
       <c r="F18" t="str">
-        <v>Submit Material Submittal (MTS) for: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
+        <v>Submit Material Submittal &amp; Compliance for: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
       </c>
       <c r="G18" t="str">
         <v>Technical Manager</v>
       </c>
       <c r="H18" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I18" t="str">
         <v>Critical</v>
@@ -1345,7 +1345,7 @@
         <v>100%</v>
       </c>
       <c r="L18" t="str">
-        <v>MTS Document Package (Status: C - Revise &amp; Resubmit)</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="19">
@@ -1353,37 +1353,37 @@
         <v>TSK-0018</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-07-26</v>
+        <v>2026-03-25</v>
       </c>
       <c r="C19" t="str">
-        <v>Engineering &amp; Approvals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D19" t="str">
-        <v>Authority Approvals</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E19" t="str">
-        <v>تقديم المخططات الأمنية وأنظمة كاميرات المراقبة لاعتماد الهيئة العليا للأمن الصناعي / MOI</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
       </c>
       <c r="F19" t="str">
-        <v>Submit Security &amp; CCTV Design package for MOI / High Commission for Industrial Security Approval</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
       </c>
       <c r="G19" t="str">
-        <v>QA/QC Director</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H19" t="str">
-        <v>All Facilities</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I19" t="str">
         <v>Critical</v>
       </c>
       <c r="J19" t="str">
-        <v>Pending</v>
+        <v>Completed</v>
       </c>
       <c r="K19" t="str">
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="L19" t="str">
-        <v>MOI Security Design Clearance Certificate</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="20">
@@ -1391,37 +1391,37 @@
         <v>TSK-0019</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-07-30</v>
+        <v>2026-04-10</v>
       </c>
       <c r="C20" t="str">
-        <v>Engineering &amp; Approvals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D20" t="str">
-        <v>Authority Approvals</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E20" t="str">
-        <v>استلام وتوثيق موافقة الدفاع المدني و MOI على منظومة المراقبة وغرف التحكم الأمني</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
       </c>
       <c r="F20" t="str">
-        <v>Obtain Final MOI Security Clearance for Security Command Center (SCC)</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
       </c>
       <c r="G20" t="str">
-        <v>Project Director</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H20" t="str">
-        <v>All Facilities</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I20" t="str">
         <v>Critical</v>
       </c>
       <c r="J20" t="str">
-        <v>Pending</v>
+        <v>Completed</v>
       </c>
       <c r="K20" t="str">
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="L20" t="str">
-        <v>Official MOI Approval Letter</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="21">
@@ -1429,37 +1429,37 @@
         <v>TSK-0020</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-09-05</v>
+        <v>2026-04-10</v>
       </c>
       <c r="C21" t="str">
-        <v>Procurement &amp; POs</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D21" t="str">
-        <v>Procurement</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E21" t="str">
-        <v>مراجعة عروض الأسعار النهائية والتفاوض مع الموردين لأنظمة AV, BGM, و Traka</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
       </c>
       <c r="F21" t="str">
-        <v>Review final vendor commercial proposals for AV, BGM &amp; Traka systems</v>
+        <v>Submit Material Submittal &amp; Compliance for: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
       </c>
       <c r="G21" t="str">
-        <v>Procurement Manager</v>
+        <v>Technical Manager</v>
       </c>
       <c r="H21" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I21" t="str">
-        <v>Critical</v>
+        <v>High</v>
       </c>
       <c r="J21" t="str">
         <v>In Progress</v>
       </c>
       <c r="K21" t="str">
-        <v>50%</v>
+        <v>40%</v>
       </c>
       <c r="L21" t="str">
-        <v>Commercial Bid Evaluation &amp; Final Price Agreements</v>
+        <v>MTS Package (Status Code: C)</v>
       </c>
     </row>
     <row r="22">
@@ -1467,37 +1467,37 @@
         <v>TSK-0021</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-09-06</v>
+        <v>2026-04-12</v>
       </c>
       <c r="C22" t="str">
-        <v>Site Construction</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D22" t="str">
-        <v>First Fix - Containment</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E22" t="str">
-        <v>فحص وتثبيت حوامل ومسارات الكابلات (Cable Trays &amp; Trunking) في القبو المشترك (Basement)</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
       </c>
       <c r="F22" t="str">
-        <v>Inspect &amp; install cable trays and trunking in Common Basement</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
       </c>
       <c r="G22" t="str">
-        <v>Site Engineer ICT/SEC</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H22" t="str">
-        <v>Common Basement</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I22" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J22" t="str">
-        <v>In Progress</v>
+        <v>Completed</v>
       </c>
       <c r="K22" t="str">
-        <v>60%</v>
+        <v>100%</v>
       </c>
       <c r="L22" t="str">
-        <v>Work Inspection Request (WIR) for Basement Containment</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="23">
@@ -1505,37 +1505,37 @@
         <v>TSK-0022</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-09-08</v>
+        <v>2026-04-15</v>
       </c>
       <c r="C23" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D23" t="str">
-        <v>MTS Resubmission</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E23" t="str">
-        <v>متابعة إعادة تقديم MTS وتلافي الملاحظات لـ: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
       </c>
       <c r="F23" t="str">
-        <v>Follow up Revise &amp; Resubmit (Code C comments) for: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
+        <v>Submit Material Submittal &amp; Compliance for: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
       </c>
       <c r="G23" t="str">
-        <v>Technical Lead</v>
+        <v>Technical Manager</v>
       </c>
       <c r="H23" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I23" t="str">
         <v>Critical</v>
       </c>
       <c r="J23" t="str">
-        <v>In Progress</v>
+        <v>Completed</v>
       </c>
       <c r="K23" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="L23" t="str">
-        <v>Updated MTS Compliance Sheet &amp; Consultant Approval</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="24">
@@ -1543,37 +1543,37 @@
         <v>TSK-0023</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-09-08</v>
+        <v>2026-04-28</v>
       </c>
       <c r="C24" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D24" t="str">
-        <v>MTS Resubmission</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E24" t="str">
-        <v>متابعة إعادة تقديم MTS وتلافي الملاحظات لـ: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
       </c>
       <c r="F24" t="str">
-        <v>Follow up Revise &amp; Resubmit (Code C comments) for: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
       </c>
       <c r="G24" t="str">
-        <v>Technical Lead</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H24" t="str">
-        <v>General</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I24" t="str">
         <v>Critical</v>
       </c>
       <c r="J24" t="str">
-        <v>In Progress</v>
+        <v>Completed</v>
       </c>
       <c r="K24" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="L24" t="str">
-        <v>Updated MTS Compliance Sheet &amp; Consultant Approval</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="25">
@@ -1581,37 +1581,37 @@
         <v>TSK-0024</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-09-08</v>
+        <v>2026-05-12</v>
       </c>
       <c r="C25" t="str">
-        <v>Engineering &amp; Submittals</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D25" t="str">
-        <v>MTS Resubmission</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E25" t="str">
-        <v>متابعة إعادة تقديم MTS وتلافي الملاحظات لـ: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
       </c>
       <c r="F25" t="str">
-        <v>Follow up Revise &amp; Resubmit (Code C comments) for: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
+        <v>Submit Material Submittal &amp; Compliance for: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
       </c>
       <c r="G25" t="str">
-        <v>Technical Lead</v>
+        <v>Technical Manager</v>
       </c>
       <c r="H25" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I25" t="str">
         <v>Critical</v>
       </c>
       <c r="J25" t="str">
-        <v>In Progress</v>
+        <v>Completed</v>
       </c>
       <c r="K25" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="L25" t="str">
-        <v>Updated MTS Compliance Sheet &amp; Consultant Approval</v>
+        <v>MTS Package (Status Code: B)</v>
       </c>
     </row>
     <row r="26">
@@ -1619,37 +1619,37 @@
         <v>TSK-0025</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-09-08</v>
+        <v>2026-05-20</v>
       </c>
       <c r="C26" t="str">
-        <v>Procurement &amp; POs</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D26" t="str">
-        <v>Procurement</v>
+        <v>Material Submittal (MTS)</v>
       </c>
       <c r="E26" t="str">
-        <v>إصدار أمر الشراء (PO) لنظام إدارة المفاتيح الذكي Traka Key Management</v>
+        <v>تقديم واعتماد عينات ومواصفات مادة/نظام: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
       </c>
       <c r="F26" t="str">
-        <v>Issue Purchase Order (PO) for Traka Key Management System</v>
+        <v>Submit Material Submittal &amp; Compliance for: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
       </c>
       <c r="G26" t="str">
-        <v>Procurement Officer</v>
+        <v>Technical Manager</v>
       </c>
       <c r="H26" t="str">
-        <v>General</v>
+        <v>Engineering Office</v>
       </c>
       <c r="I26" t="str">
         <v>Critical</v>
       </c>
       <c r="J26" t="str">
-        <v>Pending</v>
+        <v>In Progress</v>
       </c>
       <c r="K26" t="str">
-        <v>0%</v>
+        <v>40%</v>
       </c>
       <c r="L26" t="str">
-        <v>Signed Purchase Order &amp; Delivery Schedule Confirmation</v>
+        <v>MTS Package (Status Code: C)</v>
       </c>
     </row>
     <row r="27">
@@ -1657,37 +1657,37 @@
         <v>TSK-0026</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-09-10</v>
+        <v>2026-06-02</v>
       </c>
       <c r="C27" t="str">
-        <v>Procurement &amp; POs</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D27" t="str">
-        <v>Procurement</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E27" t="str">
-        <v>إصدار أمر الشراء (PO) لأنظمة الصوتيات والمرئيات AV (Crestron / Bose) و BGM</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
       </c>
       <c r="F27" t="str">
-        <v>Issue Purchase Orders for AV Systems &amp; Bose BGM Packages</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
       </c>
       <c r="G27" t="str">
         <v>Procurement Manager</v>
       </c>
       <c r="H27" t="str">
-        <v>General</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I27" t="str">
         <v>Critical</v>
       </c>
       <c r="J27" t="str">
-        <v>Pending</v>
+        <v>Completed</v>
       </c>
       <c r="K27" t="str">
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="L27" t="str">
-        <v>Executed POs with Factory Dispatch Dates</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="28">
@@ -1695,37 +1695,37 @@
         <v>TSK-0027</v>
       </c>
       <c r="B28" t="str">
-        <v>2026-09-12</v>
+        <v>2026-06-18</v>
       </c>
       <c r="C28" t="str">
-        <v>Procurement &amp; POs</v>
+        <v>Engineering &amp; Procurement</v>
       </c>
       <c r="D28" t="str">
-        <v>Procurement</v>
+        <v>Purchase Order (PO)</v>
       </c>
       <c r="E28" t="str">
-        <v>إصدار أمر الشراء (PO) لأنظمة إدارة غرف النزلاء GRMS (Schneider) وأقفال الفنادق (Assa Abloy)</v>
+        <v>إصدار وتعميد أمر الشراء الرسمي (PO) لمادة/نظام: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
       </c>
       <c r="F28" t="str">
-        <v>Issue POs for GRMS (Schneider) and Hotel Door Locks (Assa Abloy)</v>
+        <v>Issue Official PO &amp; Sign Supplier Contract for: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
       </c>
       <c r="G28" t="str">
-        <v>Procurement Officer</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H28" t="str">
-        <v>H-32, H-30, H-27</v>
+        <v>Head Office / Procurement</v>
       </c>
       <c r="I28" t="str">
         <v>Critical</v>
       </c>
       <c r="J28" t="str">
-        <v>Pending</v>
+        <v>Completed</v>
       </c>
       <c r="K28" t="str">
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="L28" t="str">
-        <v>Signed POs &amp; Factory Manufacturing Slots</v>
+        <v>Issued PO Copy &amp; Confirmed Delivery Schedule</v>
       </c>
     </row>
     <row r="29">
@@ -1733,25 +1733,25 @@
         <v>TSK-0028</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-09-14</v>
+        <v>2026-07-15</v>
       </c>
       <c r="C29" t="str">
-        <v>Site Construction</v>
+        <v>Milestone Completion</v>
       </c>
       <c r="D29" t="str">
-        <v>First Fix - Cabling</v>
+        <v>QA/QC &amp; Delivery</v>
       </c>
       <c r="E29" t="str">
-        <v>بدء سحب كابلات الألياف الضوئية الرئيسية (Backbone OS2/OM4) من غرفة الـ MDF بالقبو إلى غرف الـ IDF</v>
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: نمذجة معلومات البناء وتنسيق BIM (BIM Coordination)</v>
       </c>
       <c r="F29" t="str">
-        <v>Commence Fiber Optic Backbone cabling (OS2/OM4) from MDF to IDF risers</v>
+        <v>Finalize and deliver outputs for milestone: نمذجة معلومات البناء وتنسيق BIM (BIM Coordination)</v>
       </c>
       <c r="G29" t="str">
-        <v>Sr. ICT Infra Eng</v>
+        <v>BIM Lead</v>
       </c>
       <c r="H29" t="str">
-        <v>Common Basement to Towers</v>
+        <v>Project Site</v>
       </c>
       <c r="I29" t="str">
         <v>Critical</v>
@@ -1763,7 +1763,7 @@
         <v>0%</v>
       </c>
       <c r="L29" t="str">
-        <v>Fiber Pulling Daily Log &amp; OTDR Testing Checklist</v>
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
       </c>
     </row>
     <row r="30">
@@ -1771,37 +1771,37 @@
         <v>TSK-0029</v>
       </c>
       <c r="B30" t="str">
-        <v>2026-09-15</v>
+        <v>2026-08-01</v>
       </c>
       <c r="C30" t="str">
-        <v>Procurement &amp; POs</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D30" t="str">
-        <v>Procurement</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E30" t="str">
-        <v>إصدار أمر الشراء (PO) لوحدات التغذية غير المنقطعة UPS (Eaton) وخوادم الـ CCTV (Dell/Avigilon)</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: اعتماد المخططات الأمنية من الجهات المختصة (Security Clearance)</v>
       </c>
       <c r="F30" t="str">
-        <v>Issue POs for Rack UPSs (Eaton) and CCTV Servers &amp; Storage (Dell/Avigilon)</v>
+        <v>Commence activities for milestone: اعتماد المخططات الأمنية من الجهات المختصة (Security Clearance)</v>
       </c>
       <c r="G30" t="str">
-        <v>Procurement Manager</v>
+        <v>QA/QC Director</v>
       </c>
       <c r="H30" t="str">
-        <v>Data Centers &amp; IDF Rooms</v>
+        <v>Project Site</v>
       </c>
       <c r="I30" t="str">
-        <v>Critical</v>
+        <v>High</v>
       </c>
       <c r="J30" t="str">
-        <v>Pending</v>
+        <v>Completed</v>
       </c>
       <c r="K30" t="str">
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="L30" t="str">
-        <v>Executed Vendor POs with Air/Sea Freight Confirmation</v>
+        <v>Milestone Commencement Transmittal (5%)</v>
       </c>
     </row>
     <row r="31">
@@ -1809,37 +1809,37 @@
         <v>TSK-0030</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-09-18</v>
+        <v>2026-08-15</v>
       </c>
       <c r="C31" t="str">
-        <v>Site Construction</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D31" t="str">
-        <v>Second Fix - Cabling</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E31" t="str">
-        <v>سحب كابلات الـ Cat 6A لنقاط شبكة غرف النزلاء وكاميرات الممرات بمبنى الشقق الفندقية H-27</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: تنفيذ التأسيسات والتمديدات الأولية بالقبو والبوديوم (Basement &amp; Podium First Fix)</v>
       </c>
       <c r="F31" t="str">
-        <v>Pull Cat 6A horizontal cabling for Guest Rooms &amp; Hallway CCTV in Serviced Apartments H-27</v>
+        <v>Commence activities for milestone: تنفيذ التأسيسات والتمديدات الأولية بالقبو والبوديوم (Basement &amp; Podium First Fix)</v>
       </c>
       <c r="G31" t="str">
-        <v>Site Supervisor</v>
+        <v>Construction Manager</v>
       </c>
       <c r="H31" t="str">
-        <v>Serviced Apartment (H-27)</v>
+        <v>Project Site</v>
       </c>
       <c r="I31" t="str">
         <v>High</v>
       </c>
       <c r="J31" t="str">
-        <v>Pending</v>
+        <v>In Progress</v>
       </c>
       <c r="K31" t="str">
-        <v>0%</v>
+        <v>50%</v>
       </c>
       <c r="L31" t="str">
-        <v>Cable Continuity Test Sheets for Floors 6, 7 &amp; 8</v>
+        <v>Milestone Commencement Transmittal (8%)</v>
       </c>
     </row>
     <row r="32">
@@ -1847,37 +1847,37 @@
         <v>TSK-0031</v>
       </c>
       <c r="B32" t="str">
-        <v>2026-09-20</v>
+        <v>2026-08-20</v>
       </c>
       <c r="C32" t="str">
-        <v>Procurement &amp; POs</v>
+        <v>Milestone Completion</v>
       </c>
       <c r="D32" t="str">
-        <v>Procurement</v>
+        <v>QA/QC &amp; Delivery</v>
       </c>
       <c r="E32" t="str">
-        <v>متابعة تصنيع وشحن الكابلات الهيكلية Cat6A والألياف الضوئية Belden</v>
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: اعتماد المخططات الأمنية من الجهات المختصة (Security Clearance)</v>
       </c>
       <c r="F32" t="str">
-        <v>Track manufacturing &amp; shipping logistics for Belden SCS Fiber &amp; Copper cabling</v>
+        <v>Finalize and deliver outputs for milestone: اعتماد المخططات الأمنية من الجهات المختصة (Security Clearance)</v>
       </c>
       <c r="G32" t="str">
-        <v>Procurement Officer</v>
+        <v>QA/QC Director</v>
       </c>
       <c r="H32" t="str">
-        <v>Warehouse &amp; Site</v>
+        <v>Project Site</v>
       </c>
       <c r="I32" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J32" t="str">
-        <v>Pending</v>
+        <v>Completed</v>
       </c>
       <c r="K32" t="str">
-        <v>0%</v>
+        <v>100%</v>
       </c>
       <c r="L32" t="str">
-        <v>Bill of Lading &amp; Customs Clearance Documentation</v>
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
       </c>
     </row>
     <row r="33">
@@ -1885,25 +1885,25 @@
         <v>TSK-0032</v>
       </c>
       <c r="B33" t="str">
-        <v>2026-09-25</v>
+        <v>2026-08-20</v>
       </c>
       <c r="C33" t="str">
-        <v>Site Construction</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D33" t="str">
-        <v>Second Fix - Cabling</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E33" t="str">
-        <v>سحب كابلات نقاط الواي فاي Wi-Fi 6 وتلفزيونات IPTV في الطوابق من 1 إلى 8 بفندق F1 Overlook (H-30)</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق في الموقع</v>
       </c>
       <c r="F33" t="str">
-        <v>Pull Wi-Fi 6 AP &amp; IPTV cabling across Floors 1-8 in F1 Overlook Hotel (H-30)</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
       </c>
       <c r="G33" t="str">
-        <v>Site Engineer ICT/SEC</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H33" t="str">
-        <v>F1 Overlook Hotel (H-30)</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I33" t="str">
         <v>High</v>
@@ -1915,7 +1915,7 @@
         <v>0%</v>
       </c>
       <c r="L33" t="str">
-        <v>Fluke Calibration Test Results for H-30 Floors 1-8</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="34">
@@ -1923,25 +1923,25 @@
         <v>TSK-0033</v>
       </c>
       <c r="B34" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-30</v>
       </c>
       <c r="C34" t="str">
-        <v>Site Construction</v>
+        <v>Milestone Completion</v>
       </c>
       <c r="D34" t="str">
-        <v>First Fix - Containment</v>
+        <v>QA/QC &amp; Delivery</v>
       </c>
       <c r="E34" t="str">
-        <v>استكمال مواسير وتمديدات التأسيس الأول للطوابق 15 إلى 30 بفندق السيارات الفاخرة H-32</v>
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: المخططات الهندسية واعتمادات المواد (MTS Approvals)</v>
       </c>
       <c r="F34" t="str">
-        <v>Complete First Fix conduits &amp; backboxes for Floors 15 to 30 in Luxury Hotel H-32</v>
+        <v>Finalize and deliver outputs for milestone: المخططات الهندسية واعتمادات المواد (MTS Approvals)</v>
       </c>
       <c r="G34" t="str">
-        <v>Construction Manager</v>
+        <v>Technical Manager</v>
       </c>
       <c r="H34" t="str">
-        <v>Sports Car Hotel (H-32)</v>
+        <v>Project Site</v>
       </c>
       <c r="I34" t="str">
         <v>Critical</v>
@@ -1953,7 +1953,7 @@
         <v>0%</v>
       </c>
       <c r="L34" t="str">
-        <v>Consultant Approved WIR for Upper Floors</v>
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
       </c>
     </row>
     <row r="35">
@@ -1961,25 +1961,25 @@
         <v>TSK-0034</v>
       </c>
       <c r="B35" t="str">
-        <v>2026-10-02</v>
+        <v>2026-09-01</v>
       </c>
       <c r="C35" t="str">
-        <v>Site Construction</v>
+        <v>Milestone Execution</v>
       </c>
       <c r="D35" t="str">
-        <v>Device Installation</v>
+        <v>Planning &amp; Engineering</v>
       </c>
       <c r="E35" t="str">
-        <v>تركيب وحدات التحكم بإضاءة وتكييف الغرف GRMS في وحدات المبنى H-27</v>
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: تنفيذ أعمال الأبراج والمكاتب (Tower A &amp; B Execution)</v>
       </c>
       <c r="F35" t="str">
-        <v>Install GRMS controllers, thermostats &amp; smart switches in Serviced Apartments H-27</v>
+        <v>Commence activities for milestone: تنفيذ أعمال الأبراج والمكاتب (Tower A &amp; B Execution)</v>
       </c>
       <c r="G35" t="str">
-        <v>Sr. ICT GRMS Eng</v>
+        <v>Site Engineers</v>
       </c>
       <c r="H35" t="str">
-        <v>Serviced Apartment (H-27)</v>
+        <v>Project Site</v>
       </c>
       <c r="I35" t="str">
         <v>High</v>
@@ -1991,7 +1991,7 @@
         <v>0%</v>
       </c>
       <c r="L35" t="str">
-        <v>Room-by-Room GRMS First Fix WIR Signoff</v>
+        <v>Milestone Commencement Transmittal (12%)</v>
       </c>
     </row>
     <row r="36">
@@ -1999,37 +1999,37 @@
         <v>TSK-0035</v>
       </c>
       <c r="B36" t="str">
-        <v>2026-10-15</v>
+        <v>2026-09-10</v>
       </c>
       <c r="C36" t="str">
-        <v>Site Construction</v>
+        <v>Action Items &amp; Coordination</v>
       </c>
       <c r="D36" t="str">
-        <v>Rack Dressing &amp; Passive</v>
+        <v>Coordination</v>
       </c>
       <c r="E36" t="str">
-        <v>تجهيز وترتيب كبائن الاتصالات (Rack Dressing &amp; Patching) في غرف الـ IDF بفندق F1 (H-30)</v>
+        <v>متابعة إغلاق البند المعلق: اعتماد جدول الأبواب النهائي لتمكين فريق التركيبات من إنهاء مخططات التأسيس للأقفال الذكية</v>
       </c>
       <c r="F36" t="str">
-        <v>IDF Rack Dressing, Patch Panel termination &amp; Cable Management in Hotel H-30</v>
+        <v>Resolve Action Item: Approval of finalized Door Schedule for smart biometric access locks</v>
       </c>
       <c r="G36" t="str">
-        <v>Sr. ICT Infra Eng</v>
+        <v>المالك / المطور العقاري</v>
       </c>
       <c r="H36" t="str">
-        <v>F1 Overlook Hotel (H-30)</v>
+        <v>Management</v>
       </c>
       <c r="I36" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J36" t="str">
-        <v>Pending</v>
+        <v>Critical</v>
       </c>
       <c r="K36" t="str">
-        <v>0%</v>
+        <v>25%</v>
       </c>
       <c r="L36" t="str">
-        <v>WIR for IDF Racks &amp; Labeling Verification</v>
+        <v>Action Item Resolution Report</v>
       </c>
     </row>
     <row r="37">
@@ -2037,37 +2037,37 @@
         <v>TSK-0036</v>
       </c>
       <c r="B37" t="str">
-        <v>2026-10-20</v>
+        <v>2026-09-12</v>
       </c>
       <c r="C37" t="str">
-        <v>Site Construction</v>
+        <v>Action Items &amp; Coordination</v>
       </c>
       <c r="D37" t="str">
-        <v>Perimeter Security</v>
+        <v>Coordination</v>
       </c>
       <c r="E37" t="str">
-        <v>تركيب الحواجز الهيدروليكية (Bollards) وبوابات فحص أسفل المركبات (UVSS) وكاميرات ANPR في المداخل</v>
+        <v>متابعة إغلاق البند المعلق: إعادة التحقق من نسب إشغال مجاري الكابلات (Trunking Fill Ratio) بناءً على مخططات IFC المعتمدة</v>
       </c>
       <c r="F37" t="str">
-        <v>Install OPTIMA Hydraulic Bollards, UVSS vehicle scanners &amp; ANPR cameras at Main Gates</v>
+        <v>Resolve Action Item: Final verification of cable tray fill ratios based on latest IFC design</v>
       </c>
       <c r="G37" t="str">
-        <v>Sr. SEC Eng</v>
+        <v>استشاري المشروع / فريق التصميم</v>
       </c>
       <c r="H37" t="str">
-        <v>External Works &amp; Gates</v>
+        <v>Management</v>
       </c>
       <c r="I37" t="str">
-        <v>Critical</v>
+        <v>High</v>
       </c>
       <c r="J37" t="str">
-        <v>Pending</v>
+        <v>Open</v>
       </c>
       <c r="K37" t="str">
-        <v>0%</v>
+        <v>25%</v>
       </c>
       <c r="L37" t="str">
-        <v>WIR for Perimeter Security Infrastructure &amp; Civil Interfacing</v>
+        <v>Action Item Resolution Report</v>
       </c>
     </row>
     <row r="38">
@@ -2075,37 +2075,37 @@
         <v>TSK-0037</v>
       </c>
       <c r="B38" t="str">
-        <v>2026-11-01</v>
+        <v>2026-09-15</v>
       </c>
       <c r="C38" t="str">
-        <v>Site Construction</v>
+        <v>Action Items &amp; Coordination</v>
       </c>
       <c r="D38" t="str">
-        <v>Device Installation</v>
+        <v>Coordination</v>
       </c>
       <c r="E38" t="str">
-        <v>بدء تركيب الكاميرات الأمنية، وحساسات الحركة، وأقفال Assa Abloy الذكية في فندق H-32</v>
+        <v>متابعة إغلاق البند المعلق: إصدار أوامر الشراء الرسمية للمواد ذات فترات التوريد الطويلة (8-12 أسبوع) بعد حصر الكميات النهائي</v>
       </c>
       <c r="F38" t="str">
-        <v>Commence CCTV cameras, motion sensors &amp; Assa Abloy smart locks installation in H-32</v>
+        <v>Resolve Action Item: Release POs for Long Lead items based on approved Quantity Take-Off</v>
       </c>
       <c r="G38" t="str">
-        <v>Sr. SEC Eng</v>
+        <v>إدارة المشتريات والعقود</v>
       </c>
       <c r="H38" t="str">
-        <v>Sports Car Hotel (H-32)</v>
+        <v>Management</v>
       </c>
       <c r="I38" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J38" t="str">
-        <v>Pending</v>
+        <v>Critical</v>
       </c>
       <c r="K38" t="str">
-        <v>0%</v>
+        <v>25%</v>
       </c>
       <c r="L38" t="str">
-        <v>Device Mounting Inspection &amp; Serial Number Barcode Register</v>
+        <v>Action Item Resolution Report</v>
       </c>
     </row>
     <row r="39">
@@ -2113,37 +2113,37 @@
         <v>TSK-0038</v>
       </c>
       <c r="B39" t="str">
-        <v>2026-11-15</v>
+        <v>2026-09-18</v>
       </c>
       <c r="C39" t="str">
-        <v>Site Construction</v>
+        <v>Action Items &amp; Coordination</v>
       </c>
       <c r="D39" t="str">
-        <v>AV &amp; Systems</v>
+        <v>Coordination</v>
       </c>
       <c r="E39" t="str">
-        <v>تركيب شاشات العرض الرقمية وأنظمة الصوت BGM Bose في صالات الاستقبال والمطاعم ببرج H-32</v>
+        <v>متابعة إغلاق البند المعلق: تقديم خطط الفحص والاختبار (ITP) وطرق العمل (MOS) لغرف الخوادم وشبكات الألياف</v>
       </c>
       <c r="F39" t="str">
-        <v>Install Digital Signage screens &amp; Bose BGM ceiling speakers in H-32 Lobby &amp; Restaurants</v>
+        <v>Resolve Action Item: Method Statements (MOS) and Inspection Plans (ITP) submission</v>
       </c>
       <c r="G39" t="str">
-        <v>Sr. AVL Eng</v>
+        <v>المقاول المنفذ (مدير الجودة)</v>
       </c>
       <c r="H39" t="str">
-        <v>Sports Car Hotel (H-32)</v>
+        <v>Management</v>
       </c>
       <c r="I39" t="str">
         <v>High</v>
       </c>
       <c r="J39" t="str">
-        <v>Pending</v>
+        <v>In Progress</v>
       </c>
       <c r="K39" t="str">
-        <v>0%</v>
+        <v>25%</v>
       </c>
       <c r="L39" t="str">
-        <v>AV &amp; Sound Pressure Level (SPL) Acoustic Check Report</v>
+        <v>Action Item Resolution Report</v>
       </c>
     </row>
     <row r="40">
@@ -2151,25 +2151,25 @@
         <v>TSK-0039</v>
       </c>
       <c r="B40" t="str">
-        <v>2026-11-20</v>
+        <v>2026-10-15</v>
       </c>
       <c r="C40" t="str">
-        <v>Testing &amp; Commissioning</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D40" t="str">
-        <v>Power-On &amp; Active Config</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E40" t="str">
-        <v>إطلاق التيار الكهربائي الدائم وتشغيل وحدات الـ UPS ومفاتيح الشبكة الأساسية (HPE Aruba Core Switches)</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks في الموقع</v>
       </c>
       <c r="F40" t="str">
-        <v>Permanent Power energization, UPS commissioning &amp; Aruba Core Switch configuration</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: أقفال الأبواب الذكية وبطاقات الوصول RFID Smart Locks</v>
       </c>
       <c r="G40" t="str">
-        <v>Sr. ICT Active Eng</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H40" t="str">
-        <v>Central MDF &amp; Server Rooms</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I40" t="str">
         <v>Critical</v>
@@ -2181,7 +2181,7 @@
         <v>0%</v>
       </c>
       <c r="L40" t="str">
-        <v>Core Network Configuration Backup &amp; Ping Test Sign-off</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="41">
@@ -2189,25 +2189,25 @@
         <v>TSK-0040</v>
       </c>
       <c r="B41" t="str">
-        <v>2026-12-05</v>
+        <v>2026-10-20</v>
       </c>
       <c r="C41" t="str">
-        <v>Testing &amp; Commissioning</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D41" t="str">
-        <v>Systems Integration</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E41" t="str">
-        <v>برمجة ودمج كاميرات المراقبة مع نظام إدارة الفيديو Avigilon VMS وخوادم التخزين Dell</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: نظام الموسيقى والإذاعة الصوتية العامة BGM Package في الموقع</v>
       </c>
       <c r="F41" t="str">
-        <v>Configure CCTV Camera streams on Avigilon VMS &amp; Dell Storage NVRs with 120-day retention</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
       </c>
       <c r="G41" t="str">
-        <v>Sr. SEC Eng</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H41" t="str">
-        <v>Security Command Center (SCC)</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I41" t="str">
         <v>Critical</v>
@@ -2219,7 +2219,7 @@
         <v>0%</v>
       </c>
       <c r="L41" t="str">
-        <v>VMS Recording &amp; Live Video Analytics Verification Report</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="42">
@@ -2227,28 +2227,28 @@
         <v>TSK-0041</v>
       </c>
       <c r="B42" t="str">
-        <v>2026-12-20</v>
+        <v>2026-10-25</v>
       </c>
       <c r="C42" t="str">
-        <v>Testing &amp; Commissioning</v>
+        <v>Milestone Completion</v>
       </c>
       <c r="D42" t="str">
-        <v>GRMS &amp; BMS Integration</v>
+        <v>QA/QC &amp; Delivery</v>
       </c>
       <c r="E42" t="str">
-        <v>اختبار وتكامل نظام إدارة الغرف الذكية GRMS مع نظام إدارة المباني BMS ونظام إدارة الفندق PMS (Opera)</v>
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: إصدار أوامر الشراء للمواد طويلة التوريد (Procurement Long-Lead POs)</v>
       </c>
       <c r="F42" t="str">
-        <v>Test GRMS integration with Hotel PMS (Opera) and Schneider BMS</v>
+        <v>Finalize and deliver outputs for milestone: إصدار أوامر الشراء للمواد طويلة التوريد (Procurement Long-Lead POs)</v>
       </c>
       <c r="G42" t="str">
-        <v>Sr. ICT GRMS Eng</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H42" t="str">
-        <v>All 322 Guest Rooms</v>
+        <v>Project Site</v>
       </c>
       <c r="I42" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J42" t="str">
         <v>Pending</v>
@@ -2257,7 +2257,7 @@
         <v>0%</v>
       </c>
       <c r="L42" t="str">
-        <v>PMS Check-in / Check-out &amp; Room Climate Automation Protocol Test</v>
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
       </c>
     </row>
     <row r="43">
@@ -2265,28 +2265,28 @@
         <v>TSK-0042</v>
       </c>
       <c r="B43" t="str">
-        <v>2027-01-10</v>
+        <v>2026-10-25</v>
       </c>
       <c r="C43" t="str">
-        <v>Testing &amp; Commissioning</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D43" t="str">
-        <v>AV &amp; Sound Tuning</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E43" t="str">
-        <v>معايرة أنظمة الصوت والمؤتمرات Crestron في قاعات الاجتماعات والفعاليات بفندق H-32 و H-30</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: منظومة الهواتف والاتصال المؤسسي IP-Telephony في الموقع</v>
       </c>
       <c r="F43" t="str">
-        <v>Acoustic Tuning &amp; Crestron Conference Room commissioning in H-32 &amp; H-30 event halls</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
       </c>
       <c r="G43" t="str">
-        <v>Sr. AVL Eng</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H43" t="str">
-        <v>Meeting &amp; Event Rooms</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I43" t="str">
-        <v>Medium</v>
+        <v>Critical</v>
       </c>
       <c r="J43" t="str">
         <v>Pending</v>
@@ -2295,7 +2295,7 @@
         <v>0%</v>
       </c>
       <c r="L43" t="str">
-        <v>Audio DSP Calibration &amp; Video Wall Matrix Test Results</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="44">
@@ -2303,25 +2303,25 @@
         <v>TSK-0043</v>
       </c>
       <c r="B44" t="str">
-        <v>2027-01-25</v>
+        <v>2026-10-28</v>
       </c>
       <c r="C44" t="str">
-        <v>Testing &amp; Commissioning</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D44" t="str">
-        <v>Authority Inspection</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E44" t="str">
-        <v>فحص ومعاينة ممثلي الهيئة العليا للأمن الصناعي / MOI للمنظومة الأمنية بالموقع والحصول على الاعتماد النهائي</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: وحدات التغذية الكهربائية غير المنقطعة UPS Systems في الموقع</v>
       </c>
       <c r="F44" t="str">
-        <v>Conduct Final MOI / Security Authority on-site inspection for compliance certificate</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: وحدات التغذية الكهربائية غير المنقطعة UPS Systems</v>
       </c>
       <c r="G44" t="str">
-        <v>QA/QC Director</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H44" t="str">
-        <v>All Facilities</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I44" t="str">
         <v>Critical</v>
@@ -2333,7 +2333,7 @@
         <v>0%</v>
       </c>
       <c r="L44" t="str">
-        <v>MOI Official Inspection Sign-off &amp; System Handover Acceptance</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="45">
@@ -2341,25 +2341,25 @@
         <v>TSK-0044</v>
       </c>
       <c r="B45" t="str">
-        <v>2027-02-15</v>
+        <v>2026-10-30</v>
       </c>
       <c r="C45" t="str">
-        <v>Testing &amp; Commissioning</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D45" t="str">
-        <v>Interface &amp; Integration</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E45" t="str">
-        <v>إجراء اختبار التكامل الشامل لجميع أنظمة الـ ELV مع أنظمة إنذار الحريق وإدارة المبنى (Master Cause &amp; Effect Matrix)</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: أنظمة الصوتيات والمرئيات الاحترافية AV Systems في الموقع</v>
       </c>
       <c r="F45" t="str">
-        <v>Execute Integrated Cause &amp; Effect testing across all ELV, Fire Alarm &amp; BMS systems</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
       </c>
       <c r="G45" t="str">
-        <v>Technical Manager</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H45" t="str">
-        <v>Entire Complex</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I45" t="str">
         <v>Critical</v>
@@ -2371,7 +2371,7 @@
         <v>0%</v>
       </c>
       <c r="L45" t="str">
-        <v>Integrated Systems Testing &amp; Commissioning Certificate</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="46">
@@ -2379,28 +2379,28 @@
         <v>TSK-0045</v>
       </c>
       <c r="B46" t="str">
-        <v>2027-02-20</v>
+        <v>2026-11-01</v>
       </c>
       <c r="C46" t="str">
-        <v>Closing Out &amp; Handover</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D46" t="str">
-        <v>Documentation</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E46" t="str">
-        <v>تقديم المخططات المنفذة على الطبيعة (As-Built Drawings) وكتيبات التشغيل والصيانة (O&amp;M Manuals)</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS في الموقع</v>
       </c>
       <c r="F46" t="str">
-        <v>Submit complete As-Built Drawings, Asset Registers &amp; O&amp;M Manuals to Consultant</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS</v>
       </c>
       <c r="G46" t="str">
-        <v>Document Controller</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H46" t="str">
-        <v>All Facilities</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I46" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J46" t="str">
         <v>Pending</v>
@@ -2409,7 +2409,7 @@
         <v>0%</v>
       </c>
       <c r="L46" t="str">
-        <v>Approved As-Built &amp; O&amp;M Manuals Transmittal</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="47">
@@ -2417,28 +2417,28 @@
         <v>TSK-0046</v>
       </c>
       <c r="B47" t="str">
-        <v>2027-02-25</v>
+        <v>2026-11-01</v>
       </c>
       <c r="C47" t="str">
-        <v>Closing Out &amp; Handover</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D47" t="str">
-        <v>Training</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E47" t="str">
-        <v>تنفيذ البرنامج التدريبي الشامل لفريق تشغيل الفندق والقدية على كافة الأنظمة (Client Training)</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches في الموقع</v>
       </c>
       <c r="F47" t="str">
-        <v>Deliver comprehensive Client &amp; Operator training program for all ELV &amp; IT systems</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: مفاتيح الشبكات والموجهات الأساسية Core &amp; Edge Network Switches</v>
       </c>
       <c r="G47" t="str">
-        <v>Technical Manager</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H47" t="str">
-        <v>Hotel Training Room</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I47" t="str">
-        <v>High</v>
+        <v>Critical</v>
       </c>
       <c r="J47" t="str">
         <v>Pending</v>
@@ -2447,7 +2447,7 @@
         <v>0%</v>
       </c>
       <c r="L47" t="str">
-        <v>Signed Training Attendance Sheets &amp; Video Recorded Sessions</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="48">
@@ -2455,25 +2455,25 @@
         <v>TSK-0047</v>
       </c>
       <c r="B48" t="str">
-        <v>2027-02-28</v>
+        <v>2026-11-05</v>
       </c>
       <c r="C48" t="str">
-        <v>Closing Out &amp; Handover</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D48" t="str">
-        <v>Spare Parts &amp; Snagging</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E48" t="str">
-        <v>تسليم قطع الغيار الموصى بها (Mandatory Spare Parts) وإغلاق قائمة الملاحظات النهائية (Snag List)</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package في الموقع</v>
       </c>
       <c r="F48" t="str">
-        <v>Handover recommended spare parts and clear all Consultant Snag List items (De-snagging)</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: شاشات العرض وجدران الفيديو للمؤتمرات Video Wall Package</v>
       </c>
       <c r="G48" t="str">
-        <v>QA/QC Engineer</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H48" t="str">
-        <v>All Buildings</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I48" t="str">
         <v>Critical</v>
@@ -2485,7 +2485,7 @@
         <v>0%</v>
       </c>
       <c r="L48" t="str">
-        <v>Signed Spare Parts Handover Voucher &amp; De-Snagging Certificate</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
       </c>
     </row>
     <row r="49">
@@ -2493,25 +2493,25 @@
         <v>TSK-0048</v>
       </c>
       <c r="B49" t="str">
-        <v>2027-03-03</v>
+        <v>2026-11-05</v>
       </c>
       <c r="C49" t="str">
-        <v>Closing Out &amp; Handover</v>
+        <v>Site Delivery &amp; Logistics</v>
       </c>
       <c r="D49" t="str">
-        <v>Final Handover</v>
+        <v>Material Receiving</v>
       </c>
       <c r="E49" t="str">
-        <v>توقيع محضر الاستلام الابتدائي للمشروع (Taking-Over Certificate / TOC) وتدشين التشغيل الفعلي</v>
+        <v>وصول واستلام وفحص توريدات مادة/نظام: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage في الموقع</v>
       </c>
       <c r="F49" t="str">
-        <v>Sign Official Taking-Over Certificate (TOC) &amp; Project Commercial Handover</v>
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
       </c>
       <c r="G49" t="str">
-        <v>Project Director</v>
+        <v>Procurement Manager</v>
       </c>
       <c r="H49" t="str">
-        <v>Entire Complex (Qiddiya MSHC)</v>
+        <v>Main Warehouse / Site</v>
       </c>
       <c r="I49" t="str">
         <v>Critical</v>
@@ -2523,12 +2523,468 @@
         <v>0%</v>
       </c>
       <c r="L49" t="str">
-        <v>Signed Taking-Over Certificate (TOC) &amp; DLP Commencement</v>
+        <v>Material Inspection Request (MIR) Sign-off</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TSK-0049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>2026-11-10</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Site Delivery &amp; Logistics</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Material Receiving</v>
+      </c>
+      <c r="E50" t="str">
+        <v>وصول واستلام وفحص توريدات مادة/نظام: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka في الموقع</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Procurement Manager</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Main Warehouse / Site</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K50" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Material Inspection Request (MIR) Sign-off</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TSK-0050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>2026-11-20</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Site Delivery &amp; Logistics</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Material Receiving</v>
+      </c>
+      <c r="E51" t="str">
+        <v>وصول واستلام وفحص توريدات مادة/نظام: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers في الموقع</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Site Delivery &amp; Material Inspection Request (MIR) for: حواجز المداخل الهيدروليكية وبوابات المركبات Security Barriers</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Procurement Manager</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Main Warehouse / Site</v>
+      </c>
+      <c r="I51" t="str">
+        <v>High</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K51" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Material Inspection Request (MIR) Sign-off</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TSK-0051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>2026-11-30</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Milestone Completion</v>
+      </c>
+      <c r="D52" t="str">
+        <v>QA/QC &amp; Delivery</v>
+      </c>
+      <c r="E52" t="str">
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: تنفيذ التأسيسات والتمديدات الأولية بالقبو والبوديوم (Basement &amp; Podium First Fix)</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Finalize and deliver outputs for milestone: تنفيذ التأسيسات والتمديدات الأولية بالقبو والبوديوم (Basement &amp; Podium First Fix)</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Construction Manager</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K52" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TSK-0052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>2026-12-01</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Milestone Execution</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Planning &amp; Engineering</v>
+      </c>
+      <c r="E53" t="str">
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: الفحص والتشغيل والتكامل بين الأنظمة (Testing, Commissioning &amp; Integration)</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Commence activities for milestone: الفحص والتشغيل والتكامل بين الأنظمة (Testing, Commissioning &amp; Integration)</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Technical Manager</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I53" t="str">
+        <v>High</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K53" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Milestone Commencement Transmittal (15%)</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TSK-0053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>2027-01-30</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Milestone Completion</v>
+      </c>
+      <c r="D54" t="str">
+        <v>QA/QC &amp; Delivery</v>
+      </c>
+      <c r="E54" t="str">
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: تنفيذ أعمال الأبراج والمكاتب (Tower A &amp; B Execution)</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Finalize and deliver outputs for milestone: تنفيذ أعمال الأبراج والمكاتب (Tower A &amp; B Execution)</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Site Engineers</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K54" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TSK-0054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>2027-03-01</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Milestone Execution</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Planning &amp; Engineering</v>
+      </c>
+      <c r="E55" t="str">
+        <v>بدء تنفيذ أنشطة المعلم الرئيسي: التسليم الابتدائي والإغلاق النهائي (Handover &amp; Final Closeout)</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Commence activities for milestone: التسليم الابتدائي والإغلاق النهائي (Handover &amp; Final Closeout)</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Project Director</v>
+      </c>
+      <c r="H55" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I55" t="str">
+        <v>High</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K55" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Milestone Commencement Transmittal (5%)</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TSK-0055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2027-03-25</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Milestone Completion</v>
+      </c>
+      <c r="D56" t="str">
+        <v>QA/QC &amp; Delivery</v>
+      </c>
+      <c r="E56" t="str">
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: الفحص والتشغيل والتكامل بين الأنظمة (Testing, Commissioning &amp; Integration)</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Finalize and deliver outputs for milestone: الفحص والتشغيل والتكامل بين الأنظمة (Testing, Commissioning &amp; Integration)</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Technical Manager</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I56" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="J56" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K56" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TSK-0056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>2027-04-15</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Milestone Completion</v>
+      </c>
+      <c r="D57" t="str">
+        <v>QA/QC &amp; Delivery</v>
+      </c>
+      <c r="E57" t="str">
+        <v>استكمال ومراجعة مخرجات وتسليمات المعلم: التسليم الابتدائي والإغلاق النهائي (Handover &amp; Final Closeout)</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Finalize and deliver outputs for milestone: التسليم الابتدائي والإغلاق النهائي (Handover &amp; Final Closeout)</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Project Director</v>
+      </c>
+      <c r="H57" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K57" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Consultant Approval &amp; Milestone Sign-off Sheet</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TSK-0057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>2027-04-15</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Site Testing &amp; Integration</v>
+      </c>
+      <c r="D58" t="str">
+        <v>شبكات الاتصالات والتيار الخفيف (ICT &amp; ELV Works)</v>
+      </c>
+      <c r="E58" t="str">
+        <v>الفحص النهائي والتشغيل التجريبي لنظام: شبكات الاتصالات والتيار الخفيف (ICT &amp; ELV Works) (شبكة الألياف الضوئية وكابلات Cat 6A فائقة السرعة، مراكز البيانات المدمجة (Edge M)</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Final Testing &amp; Commissioning for: شبكات الاتصالات والتيار الخفيف (ICT &amp; ELV Works)</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Lead Site Engineer</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I58" t="str">
+        <v>High</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K58" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L58" t="str">
+        <v>System Testing &amp; Commissioning Certificate</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TSK-0058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>2027-04-15</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Site Testing &amp; Integration</v>
+      </c>
+      <c r="D59" t="str">
+        <v>المنظومة الأمنية والتحكم بالدخول (Security &amp; ACS Works)</v>
+      </c>
+      <c r="E59" t="str">
+        <v>الفحص النهائي والتشغيل التجريبي لنظام: المنظومة الأمنية والتحكم بالدخول (Security &amp; ACS Works) (كاميرات المراقبة بدقة 4K مع تحليلات الذكاء الاصطناعي (AI CCTV)، بوابات الدخول ال)</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Final Testing &amp; Commissioning for: المنظومة الأمنية والتحكم بالدخول (Security &amp; ACS Works)</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Lead Site Engineer</v>
+      </c>
+      <c r="H59" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I59" t="str">
+        <v>High</v>
+      </c>
+      <c r="J59" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K59" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L59" t="str">
+        <v>System Testing &amp; Commissioning Certificate</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TSK-0059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>2027-04-15</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Site Testing &amp; Integration</v>
+      </c>
+      <c r="D60" t="str">
+        <v>الأنظمة السمعية والبصرية والإذاعة (AV &amp; BGM Systems)</v>
+      </c>
+      <c r="E60" t="str">
+        <v>الفحص النهائي والتشغيل التجريبي لنظام: الأنظمة السمعية والبصرية والإذاعة (AV &amp; BGM Systems) (شاشات العرض الرقمية التفاعلية وجدران الفيديو (Video Walls)، نظام الإذاعة الصوتية)</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Final Testing &amp; Commissioning for: الأنظمة السمعية والبصرية والإذاعة (AV &amp; BGM Systems)</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Lead Site Engineer</v>
+      </c>
+      <c r="H60" t="str">
+        <v>Project Site</v>
+      </c>
+      <c r="I60" t="str">
+        <v>High</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K60" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L60" t="str">
+        <v>System Testing &amp; Commissioning Certificate</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TSK-0060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>2027-04-15</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Closing Out &amp; Handover</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Final Handover</v>
+      </c>
+      <c r="E61" t="str">
+        <v>الفحص النهائي وتوقيع محضر الاستلام الابتدائي (TOC) وإغلاق مشروع: مشروع برج الأفق الذكي للأعمال والفندقة</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Final Handover, Taking-Over Certificate (TOC) Sign-off for: Horizon Smart Business Tower &amp; Luxury Suites</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Project Director</v>
+      </c>
+      <c r="H61" t="str">
+        <v>Entire Project Site</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="K61" t="str">
+        <v>0%</v>
+      </c>
+      <c r="L61" t="str">
+        <v>Signed Taking-Over Certificate (TOC) &amp; As-Built Transmittals</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2785,17 +3241,21 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:M13"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2806,13 +3266,13 @@
         <v>اسم المادة / النظام (Material Submittal)</v>
       </c>
       <c r="C1" t="str">
-        <v>تاريخ التقديم</v>
+        <v>تاريخ تقديم الاعتماد</v>
       </c>
       <c r="D1" t="str">
         <v>كود الاعتماد</v>
       </c>
       <c r="E1" t="str">
-        <v>وصف الحالة</v>
+        <v>وصف الاعتماد</v>
       </c>
       <c r="F1" t="str">
         <v>فترة التوريد (Lead Time)</v>
@@ -2821,9 +3281,21 @@
         <v>مطلوب بالموقع (Required Site)</v>
       </c>
       <c r="H1" t="str">
-        <v>حالة أمر الشراء (PO)</v>
+        <v>تاريخ طلب PO (PO Request Date)</v>
       </c>
       <c r="I1" t="str">
+        <v>تاريخ اعتماد PO (PO Approval Date)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>تاريخ إصدار PO (PO Issuance Date)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>تاريخ الحالة (Status Date)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>حالة أمر الشراء (PO Status)</v>
+      </c>
+      <c r="M1" t="str">
         <v>حرج (Critical)</v>
       </c>
     </row>
@@ -2850,9 +3322,21 @@
         <v>2026-11-10</v>
       </c>
       <c r="H2" t="str">
-        <v>Pending PO</v>
+        <v>2026-02-05</v>
       </c>
       <c r="I2" t="str">
+        <v>2026-02-22</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-03-05</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-03-05</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M2" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -2879,9 +3363,21 @@
         <v>2026-10-25</v>
       </c>
       <c r="H3" t="str">
-        <v>Pending PO</v>
+        <v>2026-03-01</v>
       </c>
       <c r="I3" t="str">
+        <v>2026-03-18</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2026-03-25</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-03-25</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M3" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -2908,9 +3404,21 @@
         <v>2026-11-05</v>
       </c>
       <c r="H4" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I4" t="str">
+        <v>-</v>
+      </c>
+      <c r="J4" t="str">
+        <v>-</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-03-15</v>
+      </c>
+      <c r="L4" t="str">
         <v>Pending Revision</v>
       </c>
-      <c r="I4" t="str">
+      <c r="M4" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -2937,9 +3445,21 @@
         <v>2026-10-30</v>
       </c>
       <c r="H5" t="str">
-        <v>Pending PO</v>
+        <v>2026-03-15</v>
       </c>
       <c r="I5" t="str">
+        <v>2026-04-02</v>
+      </c>
+      <c r="J5" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M5" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -2966,9 +3486,21 @@
         <v>2026-10-20</v>
       </c>
       <c r="H6" t="str">
-        <v>Pending PO</v>
+        <v>2026-03-20</v>
       </c>
       <c r="I6" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="J6" t="str">
+        <v>2026-04-12</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2026-04-12</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M6" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -2995,9 +3527,21 @@
         <v>2026-08-20</v>
       </c>
       <c r="H7" t="str">
+        <v>2026-01-18</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-01-25</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="L7" t="str">
         <v>Delivered to Site</v>
       </c>
-      <c r="I7" t="str">
+      <c r="M7" t="str">
         <v>عادي</v>
       </c>
     </row>
@@ -3024,9 +3568,21 @@
         <v>2026-11-01</v>
       </c>
       <c r="H8" t="str">
-        <v>Pending PO</v>
+        <v>2026-05-25</v>
       </c>
       <c r="I8" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M8" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3053,9 +3609,21 @@
         <v>2026-10-28</v>
       </c>
       <c r="H9" t="str">
-        <v>Pending PO</v>
+        <v>2026-02-12</v>
       </c>
       <c r="I9" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="J9" t="str">
+        <v>2026-03-08</v>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-03-08</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M9" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3082,9 +3650,21 @@
         <v>2026-10-15</v>
       </c>
       <c r="H10" t="str">
-        <v>Pending PO</v>
+        <v>2026-04-02</v>
       </c>
       <c r="I10" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="J10" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M10" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3111,9 +3691,21 @@
         <v>2026-11-20</v>
       </c>
       <c r="H11" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="I11" t="str">
+        <v>-</v>
+      </c>
+      <c r="J11" t="str">
+        <v>-</v>
+      </c>
+      <c r="K11" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="L11" t="str">
         <v>Under Resubmission</v>
       </c>
-      <c r="I11" t="str">
+      <c r="M11" t="str">
         <v>عادي</v>
       </c>
     </row>
@@ -3140,9 +3732,21 @@
         <v>2026-11-05</v>
       </c>
       <c r="H12" t="str">
-        <v>Pending PO</v>
+        <v>2026-05-05</v>
       </c>
       <c r="I12" t="str">
+        <v>2026-05-24</v>
+      </c>
+      <c r="J12" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Issued</v>
+      </c>
+      <c r="M12" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3169,15 +3773,27 @@
         <v>2026-11-01</v>
       </c>
       <c r="H13" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="I13" t="str">
+        <v>-</v>
+      </c>
+      <c r="J13" t="str">
+        <v>-</v>
+      </c>
+      <c r="K13" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="L13" t="str">
         <v>Under Resubmission</v>
       </c>
-      <c r="I13" t="str">
+      <c r="M13" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(financials): implement BO tracking and dynamic contract-linked cash flow engine
</commit_message>
<xml_diff>
--- a/sample_output/Horizon_Smart_Tower_Daily_Schedule.xlsx
+++ b/sample_output/Horizon_Smart_Tower_Daily_Schedule.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Milestones_المعالم" sheetId="3" r:id="rId3"/>
     <sheet name="MTS_Procurement_المشتريات" sheetId="4" r:id="rId4"/>
     <sheet name="Action_Items_القرارات_المعلقة" sheetId="5" r:id="rId5"/>
+    <sheet name="CashFlow_التدفقات_النقدية" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -3241,7 +3242,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:O13"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -3255,7 +3256,9 @@
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
     <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3290,12 +3293,18 @@
         <v>تاريخ إصدار PO (PO Issuance Date)</v>
       </c>
       <c r="K1" t="str">
-        <v>تاريخ الحالة (Status Date)</v>
+        <v>تاريخ حالة PO (PO Status Date)</v>
       </c>
       <c r="L1" t="str">
         <v>حالة أمر الشراء (PO Status)</v>
       </c>
       <c r="M1" t="str">
+        <v>تاريخ حالة BO (BO Status Date)</v>
+      </c>
+      <c r="N1" t="str">
+        <v>حالة أمر الميزانية (BO Status)</v>
+      </c>
+      <c r="O1" t="str">
         <v>حرج (Critical)</v>
       </c>
     </row>
@@ -3337,6 +3346,12 @@
         <v>Issued</v>
       </c>
       <c r="M2" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O2" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3378,6 +3393,12 @@
         <v>Issued</v>
       </c>
       <c r="M3" t="str">
+        <v>2026-03-20</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O3" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3419,6 +3440,12 @@
         <v>Pending Revision</v>
       </c>
       <c r="M4" t="str">
+        <v>2026-03-15</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Pending Revision</v>
+      </c>
+      <c r="O4" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3460,6 +3487,12 @@
         <v>Issued</v>
       </c>
       <c r="M5" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O5" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3501,6 +3534,12 @@
         <v>Issued</v>
       </c>
       <c r="M6" t="str">
+        <v>2026-04-08</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O6" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3542,6 +3581,12 @@
         <v>Delivered to Site</v>
       </c>
       <c r="M7" t="str">
+        <v>2026-01-30</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Committed</v>
+      </c>
+      <c r="O7" t="str">
         <v>عادي</v>
       </c>
     </row>
@@ -3583,6 +3628,12 @@
         <v>Issued</v>
       </c>
       <c r="M8" t="str">
+        <v>2026-06-12</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O8" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3624,6 +3675,12 @@
         <v>Issued</v>
       </c>
       <c r="M9" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O9" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3665,6 +3722,12 @@
         <v>Issued</v>
       </c>
       <c r="M10" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O10" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3706,6 +3769,12 @@
         <v>Under Resubmission</v>
       </c>
       <c r="M11" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Pending BO</v>
+      </c>
+      <c r="O11" t="str">
         <v>عادي</v>
       </c>
     </row>
@@ -3747,6 +3816,12 @@
         <v>Issued</v>
       </c>
       <c r="M12" t="str">
+        <v>2026-05-28</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="O12" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
@@ -3788,12 +3863,18 @@
         <v>Under Resubmission</v>
       </c>
       <c r="M13" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Under Revision</v>
+      </c>
+      <c r="O13" t="str">
         <v>نعم (حرج)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3931,4 +4012,1115 @@
     <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L39"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>تقرير وجدول التدفقات النقدية ومنحنى S-Curve المالي المربوط بالعقد والجدول الزمني</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>قيمة العقد / الميزانية الإجمالية:</v>
+      </c>
+      <c r="B3" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>إجمالي التدفقات الداخلة المخططة (Total Inflows):</v>
+      </c>
+      <c r="B4" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>إجمالي المصروفات والتوريد (Total Outflows):</v>
+      </c>
+      <c r="B5" t="str">
+        <v>4,320,005 SAR</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>صافي السيولة النقدية (Net Cash Flow):</v>
+      </c>
+      <c r="B6" t="str">
+        <v>1,079,995 SAR</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>صافي الربح المتوقع:</v>
+      </c>
+      <c r="B7" t="str">
+        <v>1,079,995 SAR</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>هامش الربح المستهدف:</v>
+      </c>
+      <c r="B8" t="str">
+        <v>20%</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>جدول الشروط التعاقدية للدفعات ومحفزات الاستحقاق (Contract Payment Terms):</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>رمز الدفعة</v>
+      </c>
+      <c r="B11" t="str">
+        <v>اسم الدفعة التعاقدية</v>
+      </c>
+      <c r="C11" t="str">
+        <v>شرط الاستحقاق التعاقدي (Trigger)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>المعلم المرتبط في الخطة (Linked Milestone)</v>
+      </c>
+      <c r="E11" t="str">
+        <v>النسبة %</v>
+      </c>
+      <c r="F11" t="str">
+        <v>القيمة المطبقة</v>
+      </c>
+      <c r="G11" t="str">
+        <v>المستخلص المستحق (SAR)</v>
+      </c>
+      <c r="H11" t="str">
+        <v>التاريخ المخطط</v>
+      </c>
+      <c r="I11" t="str">
+        <v>الشهر المستهدف</v>
+      </c>
+      <c r="J11" t="str">
+        <v>الحالة</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PT-01</v>
+      </c>
+      <c r="B12" t="str">
+        <v>دفعة مقدمة عند توقيع العقد (Down Payment)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>توقيع العقد والمباشرة الميدانية</v>
+      </c>
+      <c r="D12" t="str">
+        <v>انطلاق المشروع والتهيئة الميدانية (Project Mobilization)</v>
+      </c>
+      <c r="E12" t="str">
+        <v>20%</v>
+      </c>
+      <c r="F12" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+      <c r="G12">
+        <v>1080000</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2025-10</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PT-02</v>
+      </c>
+      <c r="B13" t="str">
+        <v>دفعة اعتماد وتوريد المواد للموقع (Delivery &amp; Supply)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>اعتماد وتوريد المواد ذات التوريد الحرج للموقع</v>
+      </c>
+      <c r="D13" t="str">
+        <v>إصدار أوامر الشراء للمواد طويلة التوريد (Procurement Long-Lead POs)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>30%</v>
+      </c>
+      <c r="F13" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+      <c r="G13">
+        <v>1620000</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-11-01</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2026-11</v>
+      </c>
+      <c r="J13" t="str">
+        <v>In Progress</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PT-03</v>
+      </c>
+      <c r="B14" t="str">
+        <v>دفعة إنجاز أعمال التركيبات والتشييد (Installation)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>اكتمال أعمال التركيبات للأبراج والمكاتب</v>
+      </c>
+      <c r="D14" t="str">
+        <v>تنفيذ أعمال الأبراج والمكاتب (Tower A &amp; B Execution)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>30%</v>
+      </c>
+      <c r="F14" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+      <c r="G14">
+        <v>1620000</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2027-01-30</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2027-01</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Planned</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PT-04</v>
+      </c>
+      <c r="B15" t="str">
+        <v>دفعة الفحص والتشغيل والتسليم (Testing &amp; Commissioning)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>التشغيل التجريبي والفحص والتسليم النهائي</v>
+      </c>
+      <c r="D15" t="str">
+        <v>الفحص والتشغيل والتكامل بين الأنظمة (Testing, Commissioning &amp; Integration)</v>
+      </c>
+      <c r="E15" t="str">
+        <v>15%</v>
+      </c>
+      <c r="F15" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+      <c r="G15">
+        <v>810000</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2027-03-25</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2027-03</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Planned</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>PT-05</v>
+      </c>
+      <c r="B16" t="str">
+        <v>إفراج محجوز الضمان النهائي (Retention Release)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>انتهاء فترة الضمان والتسليم النهائي</v>
+      </c>
+      <c r="D16" t="str">
+        <v>التسليم الابتدائي والإغلاق النهائي (Handover &amp; Final Closeout)</v>
+      </c>
+      <c r="E16" t="str">
+        <v>5%</v>
+      </c>
+      <c r="F16" t="str">
+        <v>5,400,000 SAR</v>
+      </c>
+      <c r="G16">
+        <v>270000</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2027-05-15</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2027-05</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Planned</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>جدول توقعات التدفقات النقدية الشهرية المربوط بالمعالم (Monthly Milestone-Linked Cash Flow):</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>الشهر (Month)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>الفترة الزمنية (Period)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>الدفعات والمعالم المستحقة (Milestones Trigger)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>العقد / الحزمة / BO المرتبط</v>
+      </c>
+      <c r="E19" t="str">
+        <v>النسبة المستحقة %</v>
+      </c>
+      <c r="F19" t="str">
+        <v>المستخلص الداخل Inflow (SAR)</v>
+      </c>
+      <c r="G19" t="str">
+        <v>المصروفات والتكاليف Outflow (SAR)</v>
+      </c>
+      <c r="H19" t="str">
+        <v>صافي التدفق الشهري Net (SAR)</v>
+      </c>
+      <c r="I19" t="str">
+        <v>التدفق التراكمي الداخل (SAR)</v>
+      </c>
+      <c r="J19" t="str">
+        <v>التكاليف التراكمية (SAR)</v>
+      </c>
+      <c r="K19" t="str">
+        <v>السيولة التراكمية Cumulative Net (SAR)</v>
+      </c>
+      <c r="L19" t="str">
+        <v>الحالة (Status)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>M01</v>
+      </c>
+      <c r="B20" t="str">
+        <v>أكتوبر ٢٠٢٥ (Oct 2025)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>دفعة مقدمة عند توقيع العقد (Down Payment) (20%)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>قيمة العقد الكلية</v>
+      </c>
+      <c r="E20" t="str">
+        <v>20%</v>
+      </c>
+      <c r="F20">
+        <v>1080000</v>
+      </c>
+      <c r="G20">
+        <v>229163</v>
+      </c>
+      <c r="H20">
+        <v>850837</v>
+      </c>
+      <c r="I20">
+        <v>1080000</v>
+      </c>
+      <c r="J20">
+        <v>229163</v>
+      </c>
+      <c r="K20">
+        <v>850837</v>
+      </c>
+      <c r="L20" t="str">
+        <v>معتمد ومفوتر</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>M02</v>
+      </c>
+      <c r="B21" t="str">
+        <v>نوفمبر ٢٠٢٥ (Nov 2025)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D21" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E21" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>119475</v>
+      </c>
+      <c r="H21">
+        <v>-119475</v>
+      </c>
+      <c r="I21">
+        <v>1080000</v>
+      </c>
+      <c r="J21">
+        <v>348638</v>
+      </c>
+      <c r="K21">
+        <v>731362</v>
+      </c>
+      <c r="L21" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>M03</v>
+      </c>
+      <c r="B22" t="str">
+        <v>ديسمبر ٢٠٢٥ (Dec 2025)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D22" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E22" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>119475</v>
+      </c>
+      <c r="H22">
+        <v>-119475</v>
+      </c>
+      <c r="I22">
+        <v>1080000</v>
+      </c>
+      <c r="J22">
+        <v>468113</v>
+      </c>
+      <c r="K22">
+        <v>611887</v>
+      </c>
+      <c r="L22" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>M04</v>
+      </c>
+      <c r="B23" t="str">
+        <v>يناير ٢٠٢٦ (Jan 2026)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D23" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E23" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>119475</v>
+      </c>
+      <c r="H23">
+        <v>-119475</v>
+      </c>
+      <c r="I23">
+        <v>1080000</v>
+      </c>
+      <c r="J23">
+        <v>587588</v>
+      </c>
+      <c r="K23">
+        <v>492412</v>
+      </c>
+      <c r="L23" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>M05</v>
+      </c>
+      <c r="B24" t="str">
+        <v>فبراير ٢٠٢٦ (Feb 2026)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D24" t="str">
+        <v>توريدات: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
+      </c>
+      <c r="E24" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>185288</v>
+      </c>
+      <c r="H24">
+        <v>-185288</v>
+      </c>
+      <c r="I24">
+        <v>1080000</v>
+      </c>
+      <c r="J24">
+        <v>772876</v>
+      </c>
+      <c r="K24">
+        <v>307124</v>
+      </c>
+      <c r="L24" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>M06</v>
+      </c>
+      <c r="B25" t="str">
+        <v>مارس ٢٠٢٦ (Mar 2026)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D25" t="str">
+        <v>توريدات: نظام إدارة المفاتيح وخزائن الحفظ الذكية – Traka، منظومة الهواتف والاتصال المؤسسي IP-Telephony</v>
+      </c>
+      <c r="E25" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>316913</v>
+      </c>
+      <c r="H25">
+        <v>-316913</v>
+      </c>
+      <c r="I25">
+        <v>1080000</v>
+      </c>
+      <c r="J25">
+        <v>1089789</v>
+      </c>
+      <c r="K25">
+        <v>-9789</v>
+      </c>
+      <c r="L25" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>M07</v>
+      </c>
+      <c r="B26" t="str">
+        <v>أبريل ٢٠٢٦ (Apr 2026)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D26" t="str">
+        <v>توريدات: أنظمة الصوتيات والمرئيات الاحترافية AV Systems، نظام الموسيقى والإذاعة الصوتية العامة BGM Package</v>
+      </c>
+      <c r="E26" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>316913</v>
+      </c>
+      <c r="H26">
+        <v>-316913</v>
+      </c>
+      <c r="I26">
+        <v>1080000</v>
+      </c>
+      <c r="J26">
+        <v>1406702</v>
+      </c>
+      <c r="K26">
+        <v>-326702</v>
+      </c>
+      <c r="L26" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>M08</v>
+      </c>
+      <c r="B27" t="str">
+        <v>مايو ٢٠٢٦ (May 2026)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D27" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E27" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>119475</v>
+      </c>
+      <c r="H27">
+        <v>-119475</v>
+      </c>
+      <c r="I27">
+        <v>1080000</v>
+      </c>
+      <c r="J27">
+        <v>1526177</v>
+      </c>
+      <c r="K27">
+        <v>-446177</v>
+      </c>
+      <c r="L27" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>M09</v>
+      </c>
+      <c r="B28" t="str">
+        <v>يونيو ٢٠٢٦ (Jun 2026)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D28" t="str">
+        <v>توريدات: نظام التحكم بإضاءة وتكييف المكاتب والغرف GRMS، كاميرات المراقبة الذكية وخوادم التخزين السحابية AI CCTV &amp; Storage</v>
+      </c>
+      <c r="E28" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>251100</v>
+      </c>
+      <c r="H28">
+        <v>-251100</v>
+      </c>
+      <c r="I28">
+        <v>1080000</v>
+      </c>
+      <c r="J28">
+        <v>1777277</v>
+      </c>
+      <c r="K28">
+        <v>-697277</v>
+      </c>
+      <c r="L28" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>M10</v>
+      </c>
+      <c r="B29" t="str">
+        <v>يوليو ٢٠٢٦ (Jul 2026)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D29" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E29" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>119475</v>
+      </c>
+      <c r="H29">
+        <v>-119475</v>
+      </c>
+      <c r="I29">
+        <v>1080000</v>
+      </c>
+      <c r="J29">
+        <v>1896752</v>
+      </c>
+      <c r="K29">
+        <v>-816752</v>
+      </c>
+      <c r="L29" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>M11</v>
+      </c>
+      <c r="B30" t="str">
+        <v>أغسطس ٢٠٢٦ (Aug 2026)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D30" t="str">
+        <v>توريدات: كابلات التيار الخفيف ومسارات التمديد المقاومة للحريق</v>
+      </c>
+      <c r="E30" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>185288</v>
+      </c>
+      <c r="H30">
+        <v>-185288</v>
+      </c>
+      <c r="I30">
+        <v>1080000</v>
+      </c>
+      <c r="J30">
+        <v>2082040</v>
+      </c>
+      <c r="K30">
+        <v>-1002040</v>
+      </c>
+      <c r="L30" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>M12</v>
+      </c>
+      <c r="B31" t="str">
+        <v>سبتمبر ٢٠٢٦ (Sep 2026)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D31" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E31" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>119475</v>
+      </c>
+      <c r="H31">
+        <v>-119475</v>
+      </c>
+      <c r="I31">
+        <v>1080000</v>
+      </c>
+      <c r="J31">
+        <v>2201515</v>
+      </c>
+      <c r="K31">
+        <v>-1121515</v>
+      </c>
+      <c r="L31" t="str">
+        <v>منتهي</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>M13</v>
+      </c>
+      <c r="B32" t="str">
+        <v>أكتوبر ٢٠٢٦ (Oct 2026)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D32" t="str">
+        <v>توريدات: منظومة الهواتف والاتصال المؤسسي IP-Telephony، أنظمة الصوتيات والمرئيات الاحترافية AV Systems</v>
+      </c>
+      <c r="E32" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>448538</v>
+      </c>
+      <c r="H32">
+        <v>-448538</v>
+      </c>
+      <c r="I32">
+        <v>1080000</v>
+      </c>
+      <c r="J32">
+        <v>2650053</v>
+      </c>
+      <c r="K32">
+        <v>-1570053</v>
+      </c>
+      <c r="L32" t="str">
+        <v>مجدول بالخطة</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>M14</v>
+      </c>
+      <c r="B33" t="str">
+        <v>نوفمبر ٢٠٢٦ (Nov 2026)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>دفعة اعتماد وتوريد المواد للموقع (Delivery &amp; Supply) (30%)</v>
+      </c>
+      <c r="D33" t="str">
+        <v>حزم المشتريات ومواد المشروع (BOs &amp; POs)</v>
+      </c>
+      <c r="E33" t="str">
+        <v>30%</v>
+      </c>
+      <c r="F33">
+        <v>1620000</v>
+      </c>
+      <c r="G33">
+        <v>624038</v>
+      </c>
+      <c r="H33">
+        <v>995962</v>
+      </c>
+      <c r="I33">
+        <v>2700000</v>
+      </c>
+      <c r="J33">
+        <v>3274091</v>
+      </c>
+      <c r="K33">
+        <v>-574091</v>
+      </c>
+      <c r="L33" t="str">
+        <v>مستحق بالمعلم التعاقدي</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>M15</v>
+      </c>
+      <c r="B34" t="str">
+        <v>ديسمبر ٢٠٢٦ (Dec 2026)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D34" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E34" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>119475</v>
+      </c>
+      <c r="H34">
+        <v>-119475</v>
+      </c>
+      <c r="I34">
+        <v>2700000</v>
+      </c>
+      <c r="J34">
+        <v>3393566</v>
+      </c>
+      <c r="K34">
+        <v>-693566</v>
+      </c>
+      <c r="L34" t="str">
+        <v>مجدول بالخطة</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>M16</v>
+      </c>
+      <c r="B35" t="str">
+        <v>يناير ٢٠٢٧ (Jan 2027)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>دفعة إنجاز أعمال التركيبات والتشييد (Installation) (30%)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>الأعمال الإنشائية والتركيبات الميدانية</v>
+      </c>
+      <c r="E35" t="str">
+        <v>30%</v>
+      </c>
+      <c r="F35">
+        <v>1620000</v>
+      </c>
+      <c r="G35">
+        <v>229163</v>
+      </c>
+      <c r="H35">
+        <v>1390837</v>
+      </c>
+      <c r="I35">
+        <v>4320000</v>
+      </c>
+      <c r="J35">
+        <v>3622729</v>
+      </c>
+      <c r="K35">
+        <v>697271</v>
+      </c>
+      <c r="L35" t="str">
+        <v>مستحق بالمعلم التعاقدي</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>M17</v>
+      </c>
+      <c r="B36" t="str">
+        <v>فبراير ٢٠٢٧ (Feb 2027)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D36" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E36" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>119475</v>
+      </c>
+      <c r="H36">
+        <v>-119475</v>
+      </c>
+      <c r="I36">
+        <v>4320000</v>
+      </c>
+      <c r="J36">
+        <v>3742204</v>
+      </c>
+      <c r="K36">
+        <v>577796</v>
+      </c>
+      <c r="L36" t="str">
+        <v>مجدول بالخطة</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>M18</v>
+      </c>
+      <c r="B37" t="str">
+        <v>مارس ٢٠٢٧ (Mar 2027)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>دفعة الفحص والتشغيل والتسليم (Testing &amp; Commissioning) (15%)</v>
+      </c>
+      <c r="D37" t="str">
+        <v>حزمة الفحص والاختبارات والتسليم</v>
+      </c>
+      <c r="E37" t="str">
+        <v>15%</v>
+      </c>
+      <c r="F37">
+        <v>810000</v>
+      </c>
+      <c r="G37">
+        <v>229163</v>
+      </c>
+      <c r="H37">
+        <v>580837</v>
+      </c>
+      <c r="I37">
+        <v>5130000</v>
+      </c>
+      <c r="J37">
+        <v>3971367</v>
+      </c>
+      <c r="K37">
+        <v>1158633</v>
+      </c>
+      <c r="L37" t="str">
+        <v>مستحق بالمعلم التعاقدي</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>M19</v>
+      </c>
+      <c r="B38" t="str">
+        <v>أبريل ٢٠٢٧ (Apr 2027)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>أعمال تنفيذية ومتابعة دورية</v>
+      </c>
+      <c r="D38" t="str">
+        <v>بنود العقد العام</v>
+      </c>
+      <c r="E38" t="str">
+        <v>0%</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>119475</v>
+      </c>
+      <c r="H38">
+        <v>-119475</v>
+      </c>
+      <c r="I38">
+        <v>5130000</v>
+      </c>
+      <c r="J38">
+        <v>4090842</v>
+      </c>
+      <c r="K38">
+        <v>1039158</v>
+      </c>
+      <c r="L38" t="str">
+        <v>مجدول بالخطة</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>M20</v>
+      </c>
+      <c r="B39" t="str">
+        <v>مايو ٢٠٢٧ (May 2027)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>إفراج محجوز الضمان النهائي (Retention Release) (5%)</v>
+      </c>
+      <c r="D39" t="str">
+        <v>محجوز الضمان التعاقدي (Contract Retention)</v>
+      </c>
+      <c r="E39" t="str">
+        <v>5%</v>
+      </c>
+      <c r="F39">
+        <v>270000</v>
+      </c>
+      <c r="G39">
+        <v>229163</v>
+      </c>
+      <c r="H39">
+        <v>40837</v>
+      </c>
+      <c r="I39">
+        <v>5400000</v>
+      </c>
+      <c r="J39">
+        <v>4320005</v>
+      </c>
+      <c r="K39">
+        <v>1079995</v>
+      </c>
+      <c r="L39" t="str">
+        <v>مستحق بالمعلم التعاقدي</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L39"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>